<commit_message>
Tegenbegroting 2027: wegenfundering WarmteStad geschrapt (post uit 2026, al uitgevoerd)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gpinc7W9kdxFe2j2GC2ZtD
</commit_message>
<xml_diff>
--- a/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
+++ b/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
@@ -477,7 +477,7 @@
         <v>130.617</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>138.662202</v>
+        <v>138.212202</v>
       </c>
       <c r="D2" s="2">
         <f>C2-B2</f>
@@ -511,7 +511,7 @@
         <v>51.475</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>24.418231</v>
+        <v>23.968231</v>
       </c>
       <c r="D4" s="2">
         <f>C4-B4</f>
@@ -2995,7 +2995,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wegenfundering Warmtestad</t>
+          <t>Route Arbeid+ niet uitbreiden</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3010,17 +3010,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>p_wegenfundering_warmtestad</t>
+          <t>p_route_arbeid_plus</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n">
-        <v>0.45</v>
+        <v>-0.35</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="J47" s="2">
         <f>I47-H47</f>
@@ -3035,12 +3035,16 @@
       <c r="M47" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Teken: in de game uitbreiding niet doorzetten (besparing), v1 als uitgave.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Route Arbeid+ niet uitbreiden</t>
+          <t>Schrappen cultuurprogramma Niemeyer</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3055,17 +3059,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>p_route_arbeid_plus</t>
+          <t>p_niemeyer</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n">
-        <v>-0.35</v>
+        <v>0.25</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="J48" s="2">
         <f>I48-H48</f>
@@ -3080,16 +3084,12 @@
       <c r="M48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>Teken: in de game uitbreiding niet doorzetten (besparing), v1 als uitgave.</t>
-        </is>
-      </c>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Schrappen cultuurprogramma Niemeyer</t>
+          <t>Stoppen uitvoering plan van aanpak diversiteit</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3104,17 +3104,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>p_niemeyer</t>
+          <t>p_diversiteit_organisatie</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n">
-        <v>0.25</v>
+        <v>0.205</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.25</v>
+        <v>0.205</v>
       </c>
       <c r="J49" s="2">
         <f>I49-H49</f>
@@ -3134,7 +3134,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Stoppen uitvoering plan van aanpak diversiteit</t>
+          <t>Organisatiekosten Energiebedrijf Groningen</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3149,17 +3149,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>p_diversiteit_organisatie</t>
+          <t>p_energiebedrijf</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n">
-        <v>0.205</v>
+        <v>0.201</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.205</v>
+        <v>0.201</v>
       </c>
       <c r="J50" s="2">
         <f>I50-H50</f>
@@ -3179,7 +3179,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Organisatiekosten Energiebedrijf Groningen</t>
+          <t>Geen gemeentegeld voor dierenartskosten</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3194,17 +3194,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>p_energiebedrijf</t>
+          <t>k_dierenarts</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n">
-        <v>0.201</v>
+        <v>0.05</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.201</v>
+        <v>0.05</v>
       </c>
       <c r="J51" s="2">
         <f>I51-H51</f>
@@ -3224,52 +3224,62 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Geen gemeentegeld voor dierenartskosten</t>
+          <t>Verlaging OZB 20%</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ombuiging</t>
+          <t>Uitgave</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>k_dierenarts</t>
+          <t>t1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" s="2" t="n"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>139.441</v>
+      </c>
       <c r="H52" s="2" t="n">
-        <v>0.05</v>
+        <v>-27.88</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.05</v>
+        <v>-27.8882</v>
       </c>
       <c r="J52" s="2">
         <f>I52-H52</f>
         <v/>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>-27.8882</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0</v>
+        <v>-27.8882</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" t="inlineStr"/>
+        <v>-27.8882</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Afronding (27,888).</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Verlaging OZB 20%</t>
+          <t>Extra investeren in beheer en onderhoud openbare ruimte 20%</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3284,7 +3294,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>t1</t>
+          <t>o1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -3294,37 +3304,33 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>139.441</v>
+        <v>70.30000000000001</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>-27.88</v>
+        <v>-14.06</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>-27.8882</v>
+        <v>-14.06</v>
       </c>
       <c r="J53" s="2">
         <f>I53-H53</f>
         <v/>
       </c>
       <c r="K53" s="2" t="n">
-        <v>-27.8882</v>
+        <v>-14.06</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>-27.8882</v>
+        <v>-14.06</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>-27.8882</v>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>Afronding (27,888).</t>
-        </is>
-      </c>
+        <v>-14.06</v>
+      </c>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Extra investeren in beheer en onderhoud openbare ruimte 20%</t>
+          <t>Kettingeffect: subsidies afbouwen kost tijd</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3339,43 +3345,45 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>o1</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>70.30000000000001</v>
-      </c>
+          <t>jur_subsidies</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n">
-        <v>-14.06</v>
+        <v>-0</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>-14.06</v>
+        <v>-13.431375</v>
       </c>
       <c r="J54" s="2">
         <f>I54-H54</f>
         <v/>
       </c>
       <c r="K54" s="2" t="n">
-        <v>-14.06</v>
+        <v>-0</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>-14.06</v>
+        <v>-0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>-14.06</v>
-      </c>
-      <c r="N54" t="inlineStr"/>
+        <v>-0</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kettingeffect: subsidies afbouwen kost tijd</t>
+          <t>Jeugdzorg 10%</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3390,45 +3398,43 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>jur_subsidies</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" s="2" t="n"/>
+          <t>z1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>125.9</v>
+      </c>
       <c r="H55" s="2" t="n">
-        <v>-0</v>
+        <v>-12.59</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>-13.431375</v>
+        <v>-12.59</v>
       </c>
       <c r="J55" s="2">
         <f>I55-H55</f>
         <v/>
       </c>
       <c r="K55" s="2" t="n">
-        <v>-0</v>
+        <v>-12.59</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>-0</v>
+        <v>-12.59</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
-        </is>
-      </c>
+        <v>-12.59</v>
+      </c>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Jeugdzorg 10%</t>
+          <t>Kettingeffect: lopende Wmo-contracten</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3443,43 +3449,45 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>z1</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>125.9</v>
-      </c>
+          <t>jur_contracten</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" s="2" t="n"/>
       <c r="H56" s="2" t="n">
-        <v>-12.59</v>
+        <v>-0</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>-12.59</v>
+        <v>-10.32</v>
       </c>
       <c r="J56" s="2">
         <f>I56-H56</f>
         <v/>
       </c>
       <c r="K56" s="2" t="n">
-        <v>-12.59</v>
+        <v>-0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>-12.59</v>
+        <v>-0</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>-12.59</v>
-      </c>
-      <c r="N56" t="inlineStr"/>
+        <v>-0</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Kettingeffect: lopende Wmo-contracten</t>
+          <t>Betaald parkeren verlagen (kortparkeren) 20%</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3494,45 +3502,45 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>jur_contracten</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
+          <t>t5:kortparkeren</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n">
-        <v>-0</v>
+        <v>-4.72</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>-10.32</v>
+        <v>-4.7269906967416</v>
       </c>
       <c r="J57" s="2">
         <f>I57-H57</f>
         <v/>
       </c>
       <c r="K57" s="2" t="n">
-        <v>-0</v>
+        <v>-4.7269906967416</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>-0</v>
+        <v>-4.7269906967416</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>-0</v>
+        <v>-4.7269906967416</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+          <t>Afronding (4,727).</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Betaald parkeren verlagen (kortparkeren) 20%</t>
+          <t>Kettingeffect: gemeenschappelijke regelingen (GGD, Regio Groningen-Assen)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3547,45 +3555,45 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>t5:kortparkeren</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>jur_gr</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n">
-        <v>-4.72</v>
+        <v>-0</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>-4.7269906967416</v>
+        <v>-2.675</v>
       </c>
       <c r="J58" s="2">
         <f>I58-H58</f>
         <v/>
       </c>
       <c r="K58" s="2" t="n">
-        <v>-4.7269906967416</v>
+        <v>-2.675</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>-4.7269906967416</v>
+        <v>-0</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>-4.7269906967416</v>
+        <v>-0</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Afronding (4,727).</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Kettingeffect: gemeenschappelijke regelingen (GGD, Regio Groningen-Assen)</t>
+          <t>Intensieve coaching, begeleiding naar werk 10%</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3600,45 +3608,43 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>jur_gr</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" s="2" t="n"/>
+          <t>s3</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>23.8</v>
+      </c>
       <c r="H59" s="2" t="n">
-        <v>-0</v>
+        <v>-2.38</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>-2.675</v>
+        <v>-2.38</v>
       </c>
       <c r="J59" s="2">
         <f>I59-H59</f>
         <v/>
       </c>
       <c r="K59" s="2" t="n">
-        <v>-2.675</v>
+        <v>-2.38</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>-0</v>
+        <v>-2.38</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
-        </is>
-      </c>
+        <v>-2.38</v>
+      </c>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Intensieve coaching, begeleiding naar werk 10%</t>
+          <t>Kettingeffect: bedrijfsafval, gemiste marge en doorlopende kosten</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3653,43 +3659,45 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>s3</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="n">
-        <v>23.8</v>
-      </c>
+          <t>kd_bedrijfsafval</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" s="2" t="n"/>
       <c r="H60" s="2" t="n">
-        <v>-2.38</v>
+        <v>-0</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>-2.38</v>
+        <v>-1.98</v>
       </c>
       <c r="J60" s="2">
         <f>I60-H60</f>
         <v/>
       </c>
       <c r="K60" s="2" t="n">
-        <v>-2.38</v>
+        <v>-1.98</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>-2.38</v>
+        <v>-1.98</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>-2.38</v>
-      </c>
-      <c r="N60" t="inlineStr"/>
+        <v>-1.98</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Kettingeffect: bedrijfsafval, gemiste marge en doorlopende kosten</t>
+          <t>Parkeergarages goedkoper 20%</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3704,45 +3712,45 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>kd_bedrijfsafval</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>t5:garages</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="G61" s="2" t="n"/>
       <c r="H61" s="2" t="n">
-        <v>-0</v>
+        <v>-1.76</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>-1.98</v>
+        <v>-1.755</v>
       </c>
       <c r="J61" s="2">
         <f>I61-H61</f>
         <v/>
       </c>
       <c r="K61" s="2" t="n">
-        <v>-1.98</v>
+        <v>-1.755</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>-1.98</v>
+        <v>-1.755</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>-1.98</v>
+        <v>-1.755</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+          <t>Afronding (1,755).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Parkeergarages goedkoper 20%</t>
+          <t>Sporthallen, zwembaden en ijsbaan 5%</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3757,45 +3765,43 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>t5:garages</t>
+          <t>k1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="n"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>27.3</v>
+      </c>
       <c r="H62" s="2" t="n">
-        <v>-1.76</v>
+        <v>-1.365</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>-1.755</v>
+        <v>-1.365</v>
       </c>
       <c r="J62" s="2">
         <f>I62-H62</f>
         <v/>
       </c>
       <c r="K62" s="2" t="n">
-        <v>-1.755</v>
+        <v>-1.365</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>-1.755</v>
+        <v>-1.365</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>-1.755</v>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>Afronding (1,755).</t>
-        </is>
-      </c>
+        <v>-1.365</v>
+      </c>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Sporthallen, zwembaden en ijsbaan 5%</t>
+          <t>Zakelijke dienstverlening (werkplaats en bedrijfsafval) 100%</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3810,43 +3816,43 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>k1</t>
+          <t>o4</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>27.3</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>-1.365</v>
+        <v>-1.2</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>-1.365</v>
+        <v>-1.2</v>
       </c>
       <c r="J63" s="2">
         <f>I63-H63</f>
         <v/>
       </c>
       <c r="K63" s="2" t="n">
-        <v>-1.365</v>
+        <v>-1.2</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>-1.365</v>
+        <v>-1.2</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>-1.365</v>
+        <v>-1.2</v>
       </c>
       <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Zakelijke dienstverlening (werkplaats en bedrijfsafval) 100%</t>
+          <t>Verlaging precariobelasting 60,7%</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3861,43 +3867,47 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>o4</t>
+          <t>t4</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>60,7</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.866</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>-1.2</v>
+        <v>-1.153</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>-1.2</v>
+        <v>-1.132662</v>
       </c>
       <c r="J64" s="2">
         <f>I64-H64</f>
         <v/>
       </c>
       <c r="K64" s="2" t="n">
-        <v>-1.2</v>
+        <v>-1.132662</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>-1.2</v>
+        <v>-1.132662</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>-1.2</v>
-      </c>
-      <c r="N64" t="inlineStr"/>
+        <v>-1.132662</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Basis: game 1,866 (Ontwerpbegroting 2027); lineair 1,9.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Verlaging precariobelasting 60,7%</t>
+          <t>Kettingeffect: restkosten na stoppen opvang ongedocumenteerden</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3912,47 +3922,45 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>t4</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>60,7</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>1.866</v>
-      </c>
+          <t>zp_ongedocumenteerden</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n">
-        <v>-1.153</v>
+        <v>-0</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="J65" s="2">
         <f>I65-H65</f>
         <v/>
       </c>
       <c r="K65" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Basis: game 1,866 (Ontwerpbegroting 2027); lineair 1,9.</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Kettingeffect: restkosten na stoppen opvang ongedocumenteerden</t>
+          <t>Afschaffen reclamebelasting</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3967,45 +3975,43 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>zp_ongedocumenteerden</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+          <t>t3</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
-      <c r="G66" s="2" t="n"/>
+      <c r="G66" s="2" t="n">
+        <v>0.98</v>
+      </c>
       <c r="H66" s="2" t="n">
-        <v>-0</v>
+        <v>-1</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="J66" s="2">
         <f>I66-H66</f>
         <v/>
       </c>
       <c r="K66" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+          <t>Basis: game 0,98; lineair 1,0.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Afschaffen reclamebelasting</t>
+          <t>Betaald parkeren verlagen vergunningen 20%</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4020,43 +4026,45 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>t3</t>
+          <t>t5:bewoners_1:tweede, t5:bewoners_1:derde_tm_vijfde, t5:bezoekers, t5:bewoners_1:binnenstad, t5:bedrijven, t5:bewoners_2:tweede, t5:maatschappelijk, t5:mantelzorg</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" s="2" t="n">
-        <v>0.98</v>
-      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n">
-        <v>-1</v>
+        <v>-0.78</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="J67" s="2">
         <f>I67-H67</f>
         <v/>
       </c>
       <c r="K67" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>Basis: game 0,98; lineair 1,0.</t>
+          <t>Afronding; som van 8 vergunningsposten in de game.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Betaald parkeren verlagen vergunningen 20%</t>
+          <t>Kettingeffect: minder parkeercontrole, minder naheffingen</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4071,45 +4079,45 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>t5:bewoners_1:tweede, t5:bewoners_1:derde_tm_vijfde, t5:bezoekers, t5:bewoners_1:binnenstad, t5:bedrijven, t5:bewoners_2:tweede, t5:maatschappelijk, t5:mantelzorg</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>vh_parkeerhandhaving</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="2" t="n">
-        <v>-0.78</v>
+        <v>-0</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="J68" s="2">
         <f>I68-H68</f>
         <v/>
       </c>
       <c r="K68" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>Afronding; som van 8 vergunningsposten in de game.</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Kettingeffect: minder parkeercontrole, minder naheffingen</t>
+          <t>Openbare orde en veiligheid (o.a. cameratoezicht) 10%</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4124,45 +4132,43 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>vh_parkeerhandhaving</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" s="2" t="n"/>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>5.7</v>
+      </c>
       <c r="H69" s="2" t="n">
-        <v>-0</v>
+        <v>-0.57</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>-0.5807840000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="J69" s="2">
         <f>I69-H69</f>
         <v/>
       </c>
       <c r="K69" s="2" t="n">
-        <v>-0.5807840000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>-0.5807840000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>-0.5807840000000001</v>
-      </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
-        </is>
-      </c>
+        <v>-0.57</v>
+      </c>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Openbare orde en veiligheid (o.a. cameratoezicht) 10%</t>
+          <t>Suikerzijde (gebiedsontwikkeling) 10%</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4177,7 +4183,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>e8</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -4187,33 +4193,33 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>5.7</v>
+        <v>4.3</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="J70" s="2">
         <f>I70-H70</f>
         <v/>
       </c>
       <c r="K70" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Suikerzijde (gebiedsontwikkeling) 10%</t>
+          <t>Extra boa’s 10%</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4228,7 +4234,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>e8</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -4238,33 +4244,33 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>4.3</v>
+        <v>3.7</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.37</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.37</v>
       </c>
       <c r="J71" s="2">
         <f>I71-H71</f>
         <v/>
       </c>
       <c r="K71" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.37</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.37</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.37</v>
       </c>
       <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Extra boa’s 10%</t>
+          <t>Ambtenaren gebiedsontwikkeling 5%</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4279,43 +4285,43 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>e10</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>3.7</v>
+        <v>7</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="J72" s="2">
         <f>I72-H72</f>
         <v/>
       </c>
       <c r="K72" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ambtenaren gebiedsontwikkeling 5%</t>
+          <t>Citymarketing en economische activiteiten 15%</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4330,43 +4336,47 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>e10</t>
+          <t>e3</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>7</v>
+        <v>2.25</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.345</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.3375</v>
       </c>
       <c r="J73" s="2">
         <f>I73-H73</f>
         <v/>
       </c>
       <c r="K73" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.3375</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.3375</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="N73" t="inlineStr"/>
+        <v>-0.3375</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Basis: game 2,25; lineair 2,3.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Citymarketing en economische activiteiten 15%</t>
+          <t>Verlaging toeristenbelasting 10%</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4381,47 +4391,47 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>e3</t>
+          <t>t2</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>2.25</v>
+        <v>2.998</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>-0.345</v>
+        <v>-0.3</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="J74" s="2">
         <f>I74-H74</f>
         <v/>
       </c>
       <c r="K74" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>Basis: game 2,25; lineair 2,3.</t>
+          <t>Afronding.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Verlaging toeristenbelasting 10%</t>
+          <t>Burgerzaken (extra) 5%</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4436,47 +4446,43 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>b1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>2.998</v>
+        <v>5.9</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>-0.3</v>
+        <v>-0.295</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>-0.2998</v>
+        <v>-0.295</v>
       </c>
       <c r="J75" s="2">
         <f>I75-H75</f>
         <v/>
       </c>
       <c r="K75" s="2" t="n">
-        <v>-0.2998</v>
+        <v>-0.295</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>-0.2998</v>
+        <v>-0.295</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>-0.2998</v>
-      </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>Afronding.</t>
-        </is>
-      </c>
+        <v>-0.295</v>
+      </c>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Burgerzaken (extra) 5%</t>
+          <t>Jeugd en veiligheid 10%</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4491,43 +4497,43 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>b1</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>5.9</v>
+        <v>2.8</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="J76" s="2">
         <f>I76-H76</f>
         <v/>
       </c>
       <c r="K76" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Jeugd en veiligheid 10%</t>
+          <t>Klantcontactcentrum (extra) 5%</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4542,43 +4548,43 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>v5</t>
+          <t>b2</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>2.8</v>
+        <v>4.1</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="J77" s="2">
         <f>I77-H77</f>
         <v/>
       </c>
       <c r="K77" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Klantcontactcentrum (extra) 5%</t>
+          <t>Leefkwaliteit (groen en spelen in wijken) 5%</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4593,7 +4599,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>b2</t>
+          <t>o6</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -4603,33 +4609,33 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="J78" s="2">
         <f>I78-H78</f>
         <v/>
       </c>
       <c r="K78" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Leefkwaliteit (groen en spelen in wijken) 5%</t>
+          <t>Ondermijning 10%</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4644,43 +4650,43 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>o6</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>4</v>
+        <v>1.4</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="J79" s="2">
         <f>I79-H79</f>
         <v/>
       </c>
       <c r="K79" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Ondermijning 10%</t>
+          <t>Toezicht op bouwen 5%</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4695,43 +4701,43 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>w10</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="J80" s="2">
         <f>I80-H80</f>
         <v/>
       </c>
       <c r="K80" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Toezicht op bouwen 5%</t>
+          <t>Sportstimulering 5%</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4746,7 +4752,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>w10</t>
+          <t>k2</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -4756,33 +4762,33 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="J81" s="2">
         <f>I81-H81</f>
         <v/>
       </c>
       <c r="K81" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Sportstimulering 5%</t>
+          <t>Extra geld wonen 5%</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4797,7 +4803,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>k2</t>
+          <t>w1</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -4807,33 +4813,37 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>1.8</v>
+        <v>1.775</v>
       </c>
       <c r="H82" s="2" t="n">
         <v>-0.09</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08875</v>
       </c>
       <c r="J82" s="2">
         <f>I82-H82</f>
         <v/>
       </c>
       <c r="K82" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08875</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08875</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="N82" t="inlineStr"/>
+        <v>-0.08875</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Afronding (0,08875).</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Extra geld wonen 5%</t>
+          <t>Bedrijventerreinen en winkelcentra 5%</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4848,7 +4858,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>w1</t>
+          <t>e6</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -4858,37 +4868,37 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>1.775</v>
+        <v>1.55</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="J83" s="2">
         <f>I83-H83</f>
         <v/>
       </c>
       <c r="K83" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>Afronding (0,08875).</t>
+          <t>Afronding (0,0775).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Bedrijventerreinen en winkelcentra 5%</t>
+          <t>Kettingeffect: preventie en jeugdzorg (vanaf 2028)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4903,47 +4913,45 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>e6</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="n">
-        <v>1.55</v>
-      </c>
+          <t>zp_preventie_jeugd</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n">
-        <v>-0.08</v>
+        <v>-0</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-0</v>
       </c>
       <c r="J84" s="2">
         <f>I84-H84</f>
         <v/>
       </c>
       <c r="K84" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-2.129775</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-4.25955</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-4.25955</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>Afronding (0,0775).</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Kettingeffect: preventie en jeugdzorg (vanaf 2028)</t>
+          <t>Kettingeffect: welzijn, bewegen en Wmo (vanaf 2028)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4958,7 +4966,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>zp_preventie_jeugd</t>
+          <t>zp_preventie_wmo</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4979,13 +4987,13 @@
         <v/>
       </c>
       <c r="K85" s="2" t="n">
-        <v>-2.129775</v>
+        <v>-0.52185</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>-4.25955</v>
+        <v>-1.0437</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>-4.25955</v>
+        <v>-1.0437</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -4996,7 +5004,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Kettingeffect: welzijn, bewegen en Wmo (vanaf 2028)</t>
+          <t>Kettingeffect: gemeentefonds (verdeelmodel, vanaf 2028)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5011,7 +5019,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>zp_preventie_wmo</t>
+          <t>rijk_verdeelmodel</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -5032,13 +5040,13 @@
         <v/>
       </c>
       <c r="K86" s="2" t="n">
-        <v>-0.52185</v>
+        <v>-0.2050648974675</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>-1.0437</v>
+        <v>-0.4784847607575</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>-1.0437</v>
+        <v>-0.656149983615</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -5049,7 +5057,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Kettingeffect: gemeentefonds (verdeelmodel, vanaf 2028)</t>
+          <t>Kettingeffect: cultuur en toeristenbelasting (vanaf 2028)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5064,7 +5072,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>rijk_verdeelmodel</t>
+          <t>ec_toerisme_cultuur</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -5085,13 +5093,13 @@
         <v/>
       </c>
       <c r="K87" s="2" t="n">
-        <v>-0.2050648974675</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>-0.4784847607575</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>-0.656149983615</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -5102,7 +5110,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Kettingeffect: cultuur en toeristenbelasting (vanaf 2028)</t>
+          <t>Kettingeffect: kaartverkoop schouwburg en toeristenbelasting (vanaf 2028)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5117,7 +5125,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ec_toerisme_cultuur</t>
+          <t>kd_schouwburg</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -5138,13 +5146,13 @@
         <v/>
       </c>
       <c r="K88" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -5155,7 +5163,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Kettingeffect: kaartverkoop schouwburg en toeristenbelasting (vanaf 2028)</t>
+          <t>Kettingeffect: meer openbare ruimte door nieuwe woningen (2030)</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5170,7 +5178,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>kd_schouwburg</t>
+          <t>or_areaal</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -5191,13 +5199,13 @@
         <v/>
       </c>
       <c r="K89" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0.0125</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -5208,7 +5216,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Kettingeffect: meer openbare ruimte door nieuwe woningen (2030)</t>
+          <t>Kettingeffect: frictiekosten minder ambtenaren</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -5218,12 +5226,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>or_areaal</t>
+          <t>org_frictie</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -5237,7 +5245,7 @@
         <v>-0</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>-0</v>
+        <v>-10.9476</v>
       </c>
       <c r="J90" s="2">
         <f>I90-H90</f>
@@ -5250,7 +5258,7 @@
         <v>-0</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>-0.0125</v>
+        <v>-0</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -5261,7 +5269,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Kettingeffect: frictiekosten minder ambtenaren</t>
+          <t>Kosten onderzoek SMR</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5276,21 +5284,17 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>org_frictie</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+          <t>k_smr_onderzoek</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" s="2" t="n"/>
       <c r="H91" s="2" t="n">
-        <v>-0</v>
+        <v>-0.5</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>-10.9476</v>
+        <v>-0.5</v>
       </c>
       <c r="J91" s="2">
         <f>I91-H91</f>
@@ -5305,21 +5309,17 @@
       <c r="M91" s="2" t="n">
         <v>-0</v>
       </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
-        </is>
-      </c>
+      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Kosten onderzoek SMR</t>
+          <t>Wegenfundering WarmteStad (vervallen)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Uitgave</t>
+          <t>Ombuiging</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -5329,32 +5329,36 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>k_smr_onderzoek</t>
+          <t>p_wegenfundering_warmtestad</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="2" t="n">
-        <v>-0.5</v>
+        <v>0.45</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J92" s="2">
         <f>I92-H92</f>
         <v/>
       </c>
       <c r="K92" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M92" s="2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="N92" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>Geschrapt op verzoek van de fractie: het betreft een post uit de begroting 2026 die al heeft plaatsgevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -5394,7 +5398,7 @@
       </c>
       <c r="N93" s="3" t="inlineStr">
         <is>
-          <t>v1: 51,475 (storting). Game: 24,418.</t>
+          <t>v1: 51,475 (storting). Game: 23,968.</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5768,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1.2174</v>
+        <v>0.7674</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>0</v>
@@ -5830,7 +5834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -5935,7 +5939,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Wegenfundering Warmtestad</t>
+          <t>Route Arbeid+ niet uitbreiden</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5944,17 +5948,21 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.45</v>
+        <v>-0.35</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>0.35</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Teken: in de game uitbreiding niet doorzetten (besparing), v1 als uitgave.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Route Arbeid+ niet uitbreiden</t>
+          <t>Schrappen cultuurprogramma Niemeyer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5963,21 +5971,17 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.35</v>
+        <v>0.25</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Teken: in de game uitbreiding niet doorzetten (besparing), v1 als uitgave.</t>
-        </is>
-      </c>
+        <v>0.25</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Schrappen cultuurprogramma Niemeyer</t>
+          <t>Stoppen uitvoering plan van aanpak diversiteit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5986,17 +5990,17 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.25</v>
+        <v>0.205</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.25</v>
+        <v>0.205</v>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Stoppen uitvoering plan van aanpak diversiteit</t>
+          <t>Organisatiekosten Energiebedrijf Groningen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6005,17 +6009,17 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.205</v>
+        <v>0.201</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.205</v>
+        <v>0.201</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Organisatiekosten Energiebedrijf Groningen</t>
+          <t>Geen gemeentegeld voor dierenartskosten</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6024,36 +6028,36 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.201</v>
+        <v>0.05</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.201</v>
+        <v>0.05</v>
       </c>
       <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Geen gemeentegeld voor dierenartskosten</t>
+          <t>Kettingeffect: frictiekosten minder ambtenaren</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ombuiging</t>
+          <t>Uitgave</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.05</v>
+        <v>-0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.05</v>
+        <v>-10.9476</v>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kettingeffect: frictiekosten minder ambtenaren</t>
+          <t>Kosten onderzoek SMR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6062,17 +6066,17 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0</v>
+        <v>-0.5</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>-10.9476</v>
+        <v>-0.5</v>
       </c>
       <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kosten onderzoek SMR</t>
+          <t>Verbeteren financiële positie (storting reserve)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6081,31 +6085,12 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.5</v>
+        <v>-51.475</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Verbeteren financiële positie (storting reserve)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Uitgave</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>-51.475</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>-24.418231</v>
-      </c>
-      <c r="E13" t="inlineStr">
+        <v>-23.968231</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Sluitpost = saldo 2027 (S + I).</t>
         </is>

</xml_diff>

<commit_message>
Tegenbegroting 2027: precario -20%, verwijzingen naar de game uit het document, controle tegen begroting 2027
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gpinc7W9kdxFe2j2GC2ZtD
</commit_message>
<xml_diff>
--- a/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
+++ b/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
@@ -494,7 +494,7 @@
         <v>79.142</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>114.243971</v>
+        <v>113.484509</v>
       </c>
       <c r="D3" s="2">
         <f>C3-B3</f>
@@ -511,7 +511,7 @@
         <v>51.475</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>23.968231</v>
+        <v>24.727693</v>
       </c>
       <c r="D4" s="2">
         <f>C4-B4</f>
@@ -528,7 +528,7 @@
         <v>65.083</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>59.76200677319118</v>
+        <v>60.52146877319118</v>
       </c>
       <c r="D5" s="2">
         <f>C5-B5</f>
@@ -545,7 +545,7 @@
         <v>79.039</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>74.25517741390117</v>
+        <v>75.01463941390116</v>
       </c>
       <c r="D6" s="2">
         <f>C6-B6</f>
@@ -562,7 +562,7 @@
         <v>92.995</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>87.50227769504367</v>
+        <v>88.26173969504369</v>
       </c>
       <c r="D7" s="2">
         <f>C7-B7</f>
@@ -3852,7 +3852,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Verlaging precariobelasting 60,7%</t>
+          <t>Kettingeffect: restkosten na stoppen opvang ongedocumenteerden</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3867,47 +3867,45 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>t4</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>60,7</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="n">
-        <v>1.866</v>
-      </c>
+          <t>zp_ongedocumenteerden</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n">
-        <v>-1.153</v>
+        <v>-0</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="J64" s="2">
         <f>I64-H64</f>
         <v/>
       </c>
       <c r="K64" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>-1.132662</v>
+        <v>-1.12</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Basis: game 1,866 (Ontwerpbegroting 2027); lineair 1,9.</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Kettingeffect: restkosten na stoppen opvang ongedocumenteerden</t>
+          <t>Afschaffen reclamebelasting</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3922,45 +3920,43 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>zp_ongedocumenteerden</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+          <t>t3</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" s="2" t="n"/>
+      <c r="G65" s="2" t="n">
+        <v>0.98</v>
+      </c>
       <c r="H65" s="2" t="n">
-        <v>-0</v>
+        <v>-1</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="J65" s="2">
         <f>I65-H65</f>
         <v/>
       </c>
       <c r="K65" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+          <t>Basis: game 0,98; lineair 1,0.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Afschaffen reclamebelasting</t>
+          <t>Betaald parkeren verlagen vergunningen 20%</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3975,43 +3971,45 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>t3</t>
+          <t>t5:bewoners_1:tweede, t5:bewoners_1:derde_tm_vijfde, t5:bezoekers, t5:bewoners_1:binnenstad, t5:bedrijven, t5:bewoners_2:tweede, t5:maatschappelijk, t5:mantelzorg</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" s="2" t="n">
-        <v>0.98</v>
-      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n">
-        <v>-1</v>
+        <v>-0.78</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="J66" s="2">
         <f>I66-H66</f>
         <v/>
       </c>
       <c r="K66" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.7778093032584001</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>Basis: game 0,98; lineair 1,0.</t>
+          <t>Afronding; som van 8 vergunningsposten in de game.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Betaald parkeren verlagen vergunningen 20%</t>
+          <t>Kettingeffect: minder parkeercontrole, minder naheffingen</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4026,45 +4024,45 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>t5:bewoners_1:tweede, t5:bewoners_1:derde_tm_vijfde, t5:bezoekers, t5:bewoners_1:binnenstad, t5:bedrijven, t5:bewoners_2:tweede, t5:maatschappelijk, t5:mantelzorg</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>vh_parkeerhandhaving</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n">
-        <v>-0.78</v>
+        <v>-0</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="J67" s="2">
         <f>I67-H67</f>
         <v/>
       </c>
       <c r="K67" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>-0.7778093032584001</v>
+        <v>-0.5807840000000001</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>Afronding; som van 8 vergunningsposten in de game.</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Kettingeffect: minder parkeercontrole, minder naheffingen</t>
+          <t>Openbare orde en veiligheid (o.a. cameratoezicht) 10%</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4079,45 +4077,43 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>vh_parkeerhandhaving</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" s="2" t="n"/>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>5.7</v>
+      </c>
       <c r="H68" s="2" t="n">
-        <v>-0</v>
+        <v>-0.57</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>-0.5807840000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="J68" s="2">
         <f>I68-H68</f>
         <v/>
       </c>
       <c r="K68" s="2" t="n">
-        <v>-0.5807840000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>-0.5807840000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>-0.5807840000000001</v>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
-        </is>
-      </c>
+        <v>-0.57</v>
+      </c>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Openbare orde en veiligheid (o.a. cameratoezicht) 10%</t>
+          <t>Suikerzijde (gebiedsontwikkeling) 10%</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4132,7 +4128,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>e8</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -4142,33 +4138,33 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>5.7</v>
+        <v>4.3</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="J69" s="2">
         <f>I69-H69</f>
         <v/>
       </c>
       <c r="K69" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>-0.57</v>
+        <v>-0.43</v>
       </c>
       <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Suikerzijde (gebiedsontwikkeling) 10%</t>
+          <t>Verlaging precariobelasting 20%</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4183,38 +4179,42 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>e8</t>
+          <t>t4</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>4.3</v>
+        <v>1.866</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>-0.43</v>
+        <v>-1.153</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.3732</v>
       </c>
       <c r="J70" s="2">
         <f>I70-H70</f>
         <v/>
       </c>
       <c r="K70" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.3732</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.3732</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>-0.43</v>
-      </c>
-      <c r="N70" t="inlineStr"/>
+        <v>-0.3732</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Percentage gewijzigd van −60,7% naar −20% (fractiebesluit); basis 1,866 (Ontwerpbegroting 2027, p. 5/275). v1: 1,153 bij −60,7%.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="N93" s="3" t="inlineStr">
         <is>
-          <t>v1: 51,475 (storting). Game: 23,968.</t>
+          <t>v1: 51,475 (storting). Game: 24,728.</t>
         </is>
       </c>
     </row>
@@ -5745,16 +5745,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>23.200831</v>
+        <v>23.960293</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>59.76200677319118</v>
+        <v>60.52146877319118</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>74.25517741390117</v>
+        <v>75.01463941390116</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>87.50227769504367</v>
+        <v>88.26173969504369</v>
       </c>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
@@ -6088,7 +6088,7 @@
         <v>-51.475</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-23.968231</v>
+        <v>-24.727693</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Tegenbegroting 2027: Lisa Middelbos, geen extra geld ambtenaren gebiedsontwikkeling
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gpinc7W9kdxFe2j2GC2ZtD
</commit_message>
<xml_diff>
--- a/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
+++ b/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
@@ -494,7 +494,7 @@
         <v>79.142</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>110.358725</v>
+        <v>110.008725</v>
       </c>
       <c r="D3" s="2">
         <f>C3-B3</f>
@@ -511,7 +511,7 @@
         <v>51.475</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>11.436477</v>
+        <v>11.786477</v>
       </c>
       <c r="D4" s="2">
         <f>C4-B4</f>
@@ -528,7 +528,7 @@
         <v>65.083</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>42.13325277319118</v>
+        <v>42.48325277319118</v>
       </c>
       <c r="D5" s="2">
         <f>C5-B5</f>
@@ -545,7 +545,7 @@
         <v>79.039</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>48.40215790990119</v>
+        <v>48.75215790990119</v>
       </c>
       <c r="D6" s="2">
         <f>C6-B6</f>
@@ -562,7 +562,7 @@
         <v>92.995</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>53.41009301243368</v>
+        <v>53.76009301243369</v>
       </c>
       <c r="D7" s="2">
         <f>C7-B7</f>
@@ -3786,7 +3786,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Ambtenaren gebiedsontwikkeling 5%</t>
+          <t>Citymarketing en economische activiteiten 15%</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3801,43 +3801,47 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>e10</t>
+          <t>e3</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>7</v>
+        <v>2.25</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.345</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.3375</v>
       </c>
       <c r="J62" s="2">
         <f>I62-H62</f>
         <v/>
       </c>
       <c r="K62" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.3375</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.3375</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="N62" t="inlineStr"/>
+        <v>-0.3375</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Basis: game 2,25; lineair 2,3.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Citymarketing en economische activiteiten 15%</t>
+          <t>Verlaging toeristenbelasting 10%</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3852,47 +3856,47 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>e3</t>
+          <t>t2</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>2.25</v>
+        <v>2.998</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>-0.345</v>
+        <v>-0.3</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="J63" s="2">
         <f>I63-H63</f>
         <v/>
       </c>
       <c r="K63" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>-0.3375</v>
+        <v>-0.2998</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Basis: game 2,25; lineair 2,3.</t>
+          <t>Afronding.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Verlaging toeristenbelasting 10%</t>
+          <t>Burgerzaken (extra) 5%</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3907,47 +3911,43 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>t2</t>
+          <t>b1</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>2.998</v>
+        <v>5.9</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>-0.3</v>
+        <v>-0.295</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>-0.2998</v>
+        <v>-0.295</v>
       </c>
       <c r="J64" s="2">
         <f>I64-H64</f>
         <v/>
       </c>
       <c r="K64" s="2" t="n">
-        <v>-0.2998</v>
+        <v>-0.295</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>-0.2998</v>
+        <v>-0.295</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>-0.2998</v>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>Afronding.</t>
-        </is>
-      </c>
+        <v>-0.295</v>
+      </c>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Burgerzaken (extra) 5%</t>
+          <t>Jeugd en veiligheid 10%</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3962,43 +3962,43 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>b1</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>5.9</v>
+        <v>2.8</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="J65" s="2">
         <f>I65-H65</f>
         <v/>
       </c>
       <c r="K65" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>-0.295</v>
+        <v>-0.28</v>
       </c>
       <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Jeugd en veiligheid 10%</t>
+          <t>Klantcontactcentrum (extra) 5%</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4013,43 +4013,43 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>v5</t>
+          <t>b2</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>2.8</v>
+        <v>4.1</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="J66" s="2">
         <f>I66-H66</f>
         <v/>
       </c>
       <c r="K66" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.205</v>
       </c>
       <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Klantcontactcentrum (extra) 5%</t>
+          <t>Leefkwaliteit (groen en spelen in wijken) 5%</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>b2</t>
+          <t>o6</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -4074,33 +4074,33 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="J67" s="2">
         <f>I67-H67</f>
         <v/>
       </c>
       <c r="K67" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Leefkwaliteit (groen en spelen in wijken) 5%</t>
+          <t>Ondermijning 10%</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4115,43 +4115,43 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>o6</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>4</v>
+        <v>1.4</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="J68" s="2">
         <f>I68-H68</f>
         <v/>
       </c>
       <c r="K68" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.14</v>
       </c>
       <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Ondermijning 10%</t>
+          <t>Toezicht op bouwen 5%</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4166,43 +4166,43 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>w10</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="J69" s="2">
         <f>I69-H69</f>
         <v/>
       </c>
       <c r="K69" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.1</v>
       </c>
       <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Toezicht op bouwen 5%</t>
+          <t>Sportstimulering 5%</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>w10</t>
+          <t>k2</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -4227,33 +4227,33 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="J70" s="2">
         <f>I70-H70</f>
         <v/>
       </c>
       <c r="K70" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.09</v>
       </c>
       <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Sportstimulering 5%</t>
+          <t>Extra geld wonen 5%</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>k2</t>
+          <t>w1</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -4278,33 +4278,37 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>1.8</v>
+        <v>1.775</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>-0.09</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08875</v>
       </c>
       <c r="J71" s="2">
         <f>I71-H71</f>
         <v/>
       </c>
       <c r="K71" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08875</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08875</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="N71" t="inlineStr"/>
+        <v>-0.08875</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Afronding (0,08875).</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Extra geld wonen 5%</t>
+          <t>Bedrijventerreinen en winkelcentra 5%</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4319,7 +4323,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>w1</t>
+          <t>e6</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -4329,37 +4333,37 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>1.775</v>
+        <v>1.55</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="J72" s="2">
         <f>I72-H72</f>
         <v/>
       </c>
       <c r="K72" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.0775</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>Afronding (0,08875).</t>
+          <t>Afronding (0,0775).</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Bedrijventerreinen en winkelcentra 5%</t>
+          <t>Kettingeffect: preventie en jeugdzorg (vanaf 2028)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4374,47 +4378,45 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>e6</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>1.55</v>
-      </c>
+          <t>zp_preventie_jeugd</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n">
-        <v>-0.08</v>
+        <v>-0</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-0</v>
       </c>
       <c r="J73" s="2">
         <f>I73-H73</f>
         <v/>
       </c>
       <c r="K73" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-2.129775</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-4.25955</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-4.25955</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>Afronding (0,0775).</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Kettingeffect: preventie en jeugdzorg (vanaf 2028)</t>
+          <t>Kettingeffect: welzijn, bewegen en Wmo (vanaf 2028)</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4429,7 +4431,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>zp_preventie_jeugd</t>
+          <t>zp_preventie_wmo</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4450,13 +4452,13 @@
         <v/>
       </c>
       <c r="K74" s="2" t="n">
-        <v>-2.129775</v>
+        <v>-0.52185</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>-4.25955</v>
+        <v>-1.0437</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>-4.25955</v>
+        <v>-1.0437</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -4467,7 +4469,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Kettingeffect: welzijn, bewegen en Wmo (vanaf 2028)</t>
+          <t>Kettingeffect: gemeentefonds (verdeelmodel, vanaf 2028)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4482,7 +4484,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>zp_preventie_wmo</t>
+          <t>rijk_verdeelmodel</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4503,13 +4505,13 @@
         <v/>
       </c>
       <c r="K75" s="2" t="n">
-        <v>-0.52185</v>
+        <v>-0.2050648974675</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>-1.0437</v>
+        <v>-0.4784847607575</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>-1.0437</v>
+        <v>-0.683549658225</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
@@ -4520,7 +4522,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Kettingeffect: gemeentefonds (verdeelmodel, vanaf 2028)</t>
+          <t>Kettingeffect: cultuur en toeristenbelasting (vanaf 2028)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4535,7 +4537,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>rijk_verdeelmodel</t>
+          <t>ec_toerisme_cultuur</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4556,13 +4558,13 @@
         <v/>
       </c>
       <c r="K76" s="2" t="n">
-        <v>-0.2050648974675</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>-0.4784847607575</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>-0.683549658225</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -4573,7 +4575,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Kettingeffect: cultuur en toeristenbelasting (vanaf 2028)</t>
+          <t>Kettingeffect: kaartverkoop schouwburg en toeristenbelasting (vanaf 2028)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4588,7 +4590,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ec_toerisme_cultuur</t>
+          <t>kd_schouwburg</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4609,13 +4611,13 @@
         <v/>
       </c>
       <c r="K77" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -4626,7 +4628,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Kettingeffect: kaartverkoop schouwburg en toeristenbelasting (vanaf 2028)</t>
+          <t>Kettingeffect: frictiekosten minder ambtenaren (eenmalig)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4636,12 +4638,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>kd_schouwburg</t>
+          <t>org_frictie</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4655,20 +4657,20 @@
         <v>-0</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>-0</v>
+        <v>-8.4026</v>
       </c>
       <c r="J78" s="2">
         <f>I78-H78</f>
         <v/>
       </c>
       <c r="K78" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -4679,7 +4681,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Kettingeffect: frictiekosten minder ambtenaren (eenmalig)</t>
+          <t>Kosten onderzoek SMR</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4694,21 +4696,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>org_frictie</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+          <t>k_smr_onderzoek</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n">
-        <v>-0</v>
+        <v>-0.5</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>-8.4026</v>
+        <v>-0.5</v>
       </c>
       <c r="J79" s="2">
         <f>I79-H79</f>
@@ -4723,21 +4721,17 @@
       <c r="M79" s="2" t="n">
         <v>-0</v>
       </c>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
-        </is>
-      </c>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Kosten onderzoek SMR</t>
+          <t>Wegenfundering WarmteStad (vervallen)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Uitgave</t>
+          <t>Ombuiging</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4745,39 +4739,39 @@
           <t>I</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>k_smr_onderzoek</t>
-        </is>
-      </c>
+      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n">
-        <v>-0.5</v>
+        <v>0.45</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J80" s="2">
         <f>I80-H80</f>
         <v/>
       </c>
       <c r="K80" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="N80" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Post uit de begroting 2026; al uitgevoerd (fractiebesluit).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Wegenfundering WarmteStad (vervallen)</t>
+          <t>Ambtenaren mobiliteit 40% (vervallen)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4787,7 +4781,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -4795,7 +4789,7 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n">
-        <v>0.45</v>
+        <v>1.32</v>
       </c>
       <c r="I81" s="2" t="n">
         <v>0</v>
@@ -4815,14 +4809,14 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>Post uit de begroting 2026; al uitgevoerd (fractiebesluit).</t>
+          <t>Dubbel met 15% minder ambtenaren; geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Ambtenaren mobiliteit 40% (vervallen)</t>
+          <t>Ambtenaren wonen 25% (vervallen)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4840,7 +4834,7 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n">
-        <v>1.32</v>
+        <v>1.225</v>
       </c>
       <c r="I82" s="2" t="n">
         <v>0</v>
@@ -4867,7 +4861,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Ambtenaren wonen 25% (vervallen)</t>
+          <t>Minder bouwregels: welstandsvrij bouwen (vervallen)</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4885,7 +4879,7 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="2" t="n">
-        <v>1.225</v>
+        <v>0.49</v>
       </c>
       <c r="I83" s="2" t="n">
         <v>0</v>
@@ -4905,14 +4899,14 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>Dubbel met 15% minder ambtenaren; geschrapt.</t>
+          <t>Besparing = minder ambtenaren wonen, dubbel met 15%; beleid blijft, bedrag geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Minder bouwregels: welstandsvrij bouwen (vervallen)</t>
+          <t>Parkeercontrole 20% (vervallen)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4930,7 +4924,7 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n">
-        <v>0.49</v>
+        <v>0.2</v>
       </c>
       <c r="I84" s="2" t="n">
         <v>0</v>
@@ -4950,14 +4944,14 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>Besparing = minder ambtenaren wonen, dubbel met 15%; beleid blijft, bedrag geschrapt.</t>
+          <t>Kost netto geld (minder naheffingen); geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Parkeercontrole 20% (vervallen)</t>
+          <t>Preventiefonds jeugd (v1 als uitgave) (vervallen)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4967,7 +4961,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -4975,7 +4969,7 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n">
-        <v>0.2</v>
+        <v>-4.509</v>
       </c>
       <c r="I85" s="2" t="n">
         <v>0</v>
@@ -4995,14 +4989,14 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>Kost netto geld (minder naheffingen); geschrapt.</t>
+          <t>Fonds liep t/m 2026 (begroting 2026); bestaat in 2027 niet meer.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Preventiefonds jeugd (v1 als uitgave) (vervallen)</t>
+          <t>Organisatiekosten Energiebedrijf Groningen (vervallen)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5020,7 +5014,7 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n">
-        <v>-4.509</v>
+        <v>0.201</v>
       </c>
       <c r="I86" s="2" t="n">
         <v>0</v>
@@ -5040,14 +5034,14 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>Fonds liep t/m 2026 (begroting 2026); bestaat in 2027 niet meer.</t>
+          <t>Intensivering 2026; niet in 2027.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Organisatiekosten Energiebedrijf Groningen (vervallen)</t>
+          <t>Schrappen cultuurprogramma Niemeyer (vervallen)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5065,7 +5059,7 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n">
-        <v>0.201</v>
+        <v>0.25</v>
       </c>
       <c r="I87" s="2" t="n">
         <v>0</v>
@@ -5085,14 +5079,14 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>Intensivering 2026; niet in 2027.</t>
+          <t>Intensivering 2026 (eenmalig); niet in 2027.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Schrappen cultuurprogramma Niemeyer (vervallen)</t>
+          <t>Stoppen uitvoering plan van aanpak diversiteit (vervallen)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5110,7 +5104,7 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n">
-        <v>0.25</v>
+        <v>0.205</v>
       </c>
       <c r="I88" s="2" t="n">
         <v>0</v>
@@ -5130,14 +5124,14 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>Intensivering 2026 (eenmalig); niet in 2027.</t>
+          <t>Intensivering 2026; niet in 2027.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Stoppen uitvoering plan van aanpak diversiteit (vervallen)</t>
+          <t>Ambtenaren gebiedsontwikkeling +5% (vervallen)</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5147,7 +5141,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -5155,7 +5149,7 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n">
-        <v>0.205</v>
+        <v>-0.35</v>
       </c>
       <c r="I89" s="2" t="n">
         <v>0</v>
@@ -5175,7 +5169,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>Intensivering 2026; niet in 2027.</t>
+          <t>Geschrapt (fractiebesluit): past niet bij de vacaturestop.</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5211,7 @@
       </c>
       <c r="N90" s="3" t="inlineStr">
         <is>
-          <t>v1: 51,475 (storting). Game: 11,436.</t>
+          <t>v1: 51,475 (storting). Game: 11,786.</t>
         </is>
       </c>
     </row>
@@ -5564,16 +5558,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>13.489077</v>
+        <v>13.839077</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>42.13325277319118</v>
+        <v>42.48325277319118</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>48.40215790990119</v>
+        <v>48.75215790990119</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>53.41009301243368</v>
+        <v>53.76009301243369</v>
       </c>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
@@ -5827,7 +5821,7 @@
         <v>-51.475</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-11.436477</v>
+        <v>-11.786477</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Tegenbegroting 2027: dekkend cameratoezicht binnenstad en stationsgebied
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gpinc7W9kdxFe2j2GC2ZtD
</commit_message>
<xml_diff>
--- a/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
+++ b/tegenbegroting/Tegenbegroting_fractie_gezamenlijk_v2.xlsx
@@ -494,7 +494,7 @@
         <v>79.142</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>110.008725</v>
+        <v>110.4141416666667</v>
       </c>
       <c r="D3" s="2">
         <f>C3-B3</f>
@@ -511,7 +511,7 @@
         <v>51.475</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>11.786477</v>
+        <v>11.38106033333333</v>
       </c>
       <c r="D4" s="2">
         <f>C4-B4</f>
@@ -528,7 +528,7 @@
         <v>65.083</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>42.48325277319118</v>
+        <v>42.08258610652452</v>
       </c>
       <c r="D5" s="2">
         <f>C5-B5</f>
@@ -545,7 +545,7 @@
         <v>79.039</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>48.75215790990119</v>
+        <v>48.35624124323452</v>
       </c>
       <c r="D6" s="2">
         <f>C6-B6</f>
@@ -562,7 +562,7 @@
         <v>92.995</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>53.76009301243369</v>
+        <v>53.36892634576702</v>
       </c>
       <c r="D7" s="2">
         <f>C7-B7</f>
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3998,7 +3998,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Klantcontactcentrum (extra) 5%</t>
+          <t>Cameratoezicht binnenstad en stationsgebied: kapitaallasten</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4013,43 +4013,37 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>b2</t>
+          <t>tb_camera_invest</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="n">
-        <v>4.1</v>
-      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.21375</v>
       </c>
       <c r="J66" s="2">
         <f>I66-H66</f>
         <v/>
       </c>
       <c r="K66" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.209</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.20425</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>-0.205</v>
+        <v>-0.1995</v>
       </c>
       <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Leefkwaliteit (groen en spelen in wijken) 5%</t>
+          <t>Klantcontactcentrum (extra) 5%</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4064,7 +4058,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>o6</t>
+          <t>b2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -4074,33 +4068,33 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.205</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.205</v>
       </c>
       <c r="J67" s="2">
         <f>I67-H67</f>
         <v/>
       </c>
       <c r="K67" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.205</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.205</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.205</v>
       </c>
       <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Ondermijning 10%</t>
+          <t>Leefkwaliteit (groen en spelen in wijken) 5%</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4115,43 +4109,43 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>o6</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>1.4</v>
+        <v>4</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.2</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.2</v>
       </c>
       <c r="J68" s="2">
         <f>I68-H68</f>
         <v/>
       </c>
       <c r="K68" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.2</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.2</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>-0.14</v>
+        <v>-0.2</v>
       </c>
       <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Toezicht op bouwen 5%</t>
+          <t>Cameratoezicht binnenstad en stationsgebied: uitkijken en onderhoud</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4166,43 +4160,37 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>w10</t>
+          <t>tb_camera_exploitatie</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.1916666666666667</v>
       </c>
       <c r="J69" s="2">
         <f>I69-H69</f>
         <v/>
       </c>
       <c r="K69" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.1916666666666667</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.1916666666666667</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.1916666666666667</v>
       </c>
       <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Sportstimulering 5%</t>
+          <t>Ondermijning 10%</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4217,43 +4205,43 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>k2</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="J70" s="2">
         <f>I70-H70</f>
         <v/>
       </c>
       <c r="K70" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Extra geld wonen 5%</t>
+          <t>Toezicht op bouwen 5%</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4268,7 +4256,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>w1</t>
+          <t>w10</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -4278,37 +4266,33 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>1.775</v>
+        <v>2</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.1</v>
       </c>
       <c r="J71" s="2">
         <f>I71-H71</f>
         <v/>
       </c>
       <c r="K71" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.1</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>-0.08875</v>
+        <v>-0.1</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>-0.08875</v>
-      </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>Afronding (0,08875).</t>
-        </is>
-      </c>
+        <v>-0.1</v>
+      </c>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Bedrijventerreinen en winkelcentra 5%</t>
+          <t>Sportstimulering 5%</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4323,7 +4307,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>e6</t>
+          <t>k2</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -4333,37 +4317,33 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>1.55</v>
+        <v>1.8</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-0.09</v>
       </c>
       <c r="J72" s="2">
         <f>I72-H72</f>
         <v/>
       </c>
       <c r="K72" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-0.09</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>-0.0775</v>
+        <v>-0.09</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>-0.0775</v>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>Afronding (0,0775).</t>
-        </is>
-      </c>
+        <v>-0.09</v>
+      </c>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Kettingeffect: preventie en jeugdzorg (vanaf 2028)</t>
+          <t>Extra geld wonen 5%</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4378,45 +4358,47 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>zp_preventie_jeugd</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" s="2" t="n"/>
+          <t>w1</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>1.775</v>
+      </c>
       <c r="H73" s="2" t="n">
-        <v>-0</v>
+        <v>-0.09</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>-0</v>
+        <v>-0.08875</v>
       </c>
       <c r="J73" s="2">
         <f>I73-H73</f>
         <v/>
       </c>
       <c r="K73" s="2" t="n">
-        <v>-2.129775</v>
+        <v>-0.08875</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>-4.25955</v>
+        <v>-0.08875</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>-4.25955</v>
+        <v>-0.08875</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+          <t>Afronding (0,08875).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Kettingeffect: welzijn, bewegen en Wmo (vanaf 2028)</t>
+          <t>Bedrijventerreinen en winkelcentra 5%</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4431,45 +4413,47 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>zp_preventie_wmo</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" s="2" t="n"/>
+          <t>e6</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>1.55</v>
+      </c>
       <c r="H74" s="2" t="n">
-        <v>-0</v>
+        <v>-0.08</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>-0</v>
+        <v>-0.0775</v>
       </c>
       <c r="J74" s="2">
         <f>I74-H74</f>
         <v/>
       </c>
       <c r="K74" s="2" t="n">
-        <v>-0.52185</v>
+        <v>-0.0775</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>-1.0437</v>
+        <v>-0.0775</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>-1.0437</v>
+        <v>-0.0775</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+          <t>Afronding (0,0775).</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Kettingeffect: gemeentefonds (verdeelmodel, vanaf 2028)</t>
+          <t>Kettingeffect: preventie en jeugdzorg (vanaf 2028)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4484,7 +4468,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>rijk_verdeelmodel</t>
+          <t>zp_preventie_jeugd</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4505,13 +4489,13 @@
         <v/>
       </c>
       <c r="K75" s="2" t="n">
-        <v>-0.2050648974675</v>
+        <v>-2.129775</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>-0.4784847607575</v>
+        <v>-4.25955</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>-0.683549658225</v>
+        <v>-4.25955</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
@@ -4522,7 +4506,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Kettingeffect: cultuur en toeristenbelasting (vanaf 2028)</t>
+          <t>Kettingeffect: welzijn, bewegen en Wmo (vanaf 2028)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4537,7 +4521,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ec_toerisme_cultuur</t>
+          <t>zp_preventie_wmo</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4558,13 +4542,13 @@
         <v/>
       </c>
       <c r="K76" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-0.52185</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-1.0437</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>-0.1591453293413174</v>
+        <v>-1.0437</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -4575,7 +4559,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Kettingeffect: kaartverkoop schouwburg en toeristenbelasting (vanaf 2028)</t>
+          <t>Kettingeffect: gemeentefonds (verdeelmodel, vanaf 2028)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4590,7 +4574,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>kd_schouwburg</t>
+          <t>rijk_verdeelmodel</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4611,13 +4595,13 @@
         <v/>
       </c>
       <c r="K77" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0.2050648974675</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0.4784847607575</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>-0.05396400000000001</v>
+        <v>-0.683549658225</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -4628,7 +4612,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Kettingeffect: frictiekosten minder ambtenaren (eenmalig)</t>
+          <t>Kettingeffect: cultuur en toeristenbelasting (vanaf 2028)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4638,12 +4622,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>org_frictie</t>
+          <t>ec_toerisme_cultuur</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4657,20 +4641,20 @@
         <v>-0</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>-8.4026</v>
+        <v>-0</v>
       </c>
       <c r="J78" s="2">
         <f>I78-H78</f>
         <v/>
       </c>
       <c r="K78" s="2" t="n">
-        <v>-0</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>-0</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>-0</v>
+        <v>-0.1591453293413174</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -4681,7 +4665,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Kosten onderzoek SMR</t>
+          <t>Kettingeffect: kaartverkoop schouwburg en toeristenbelasting (vanaf 2028)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4691,47 +4675,55 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>k_smr_onderzoek</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>kd_schouwburg</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n">
-        <v>-0.5</v>
+        <v>-0</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>-0.5</v>
+        <v>-0</v>
       </c>
       <c r="J79" s="2">
         <f>I79-H79</f>
         <v/>
       </c>
       <c r="K79" s="2" t="n">
-        <v>-0</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>-0</v>
+        <v>-0.05396400000000001</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="N79" t="inlineStr"/>
+        <v>-0.05396400000000001</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Wegenfundering WarmteStad (vervallen)</t>
+          <t>Kettingeffect: frictiekosten minder ambtenaren (eenmalig)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Ombuiging</t>
+          <t>Uitgave</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4739,84 +4731,92 @@
           <t>I</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>org_frictie</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n">
-        <v>0.45</v>
+        <v>-0</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>0</v>
+        <v>-8.4026</v>
       </c>
       <c r="J80" s="2">
         <f>I80-H80</f>
         <v/>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>Post uit de begroting 2026; al uitgevoerd (fractiebesluit).</t>
+          <t>Nieuwe regel: kettingeffect uit de game (niet in het lineaire model).</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Ambtenaren mobiliteit 40% (vervallen)</t>
+          <t>Kosten onderzoek SMR</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ombuiging</t>
+          <t>Uitgave</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>k_smr_onderzoek</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n">
-        <v>1.32</v>
+        <v>-0.5</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J81" s="2">
         <f>I81-H81</f>
         <v/>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>Dubbel met 15% minder ambtenaren; geschrapt.</t>
-        </is>
-      </c>
+        <v>-0</v>
+      </c>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Ambtenaren wonen 25% (vervallen)</t>
+          <t>Wegenfundering WarmteStad (vervallen)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -4834,7 +4834,7 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n">
-        <v>1.225</v>
+        <v>0.45</v>
       </c>
       <c r="I82" s="2" t="n">
         <v>0</v>
@@ -4854,14 +4854,14 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>Dubbel met 15% minder ambtenaren; geschrapt.</t>
+          <t>Post uit de begroting 2026; al uitgevoerd (fractiebesluit).</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Minder bouwregels: welstandsvrij bouwen (vervallen)</t>
+          <t>Ambtenaren mobiliteit 40% (vervallen)</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4879,7 +4879,7 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="2" t="n">
-        <v>0.49</v>
+        <v>1.32</v>
       </c>
       <c r="I83" s="2" t="n">
         <v>0</v>
@@ -4899,14 +4899,14 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>Besparing = minder ambtenaren wonen, dubbel met 15%; beleid blijft, bedrag geschrapt.</t>
+          <t>Dubbel met 15% minder ambtenaren; geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Parkeercontrole 20% (vervallen)</t>
+          <t>Ambtenaren wonen 25% (vervallen)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4924,7 +4924,7 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n">
-        <v>0.2</v>
+        <v>1.225</v>
       </c>
       <c r="I84" s="2" t="n">
         <v>0</v>
@@ -4944,14 +4944,14 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>Kost netto geld (minder naheffingen); geschrapt.</t>
+          <t>Dubbel met 15% minder ambtenaren; geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Preventiefonds jeugd (v1 als uitgave) (vervallen)</t>
+          <t>Minder bouwregels: welstandsvrij bouwen (vervallen)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -4969,7 +4969,7 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n">
-        <v>-4.509</v>
+        <v>0.49</v>
       </c>
       <c r="I85" s="2" t="n">
         <v>0</v>
@@ -4989,14 +4989,14 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>Fonds liep t/m 2026 (begroting 2026); bestaat in 2027 niet meer.</t>
+          <t>Besparing = minder ambtenaren wonen, dubbel met 15%; beleid blijft, bedrag geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Organisatiekosten Energiebedrijf Groningen (vervallen)</t>
+          <t>Parkeercontrole 20% (vervallen)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
@@ -5014,7 +5014,7 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n">
-        <v>0.201</v>
+        <v>0.2</v>
       </c>
       <c r="I86" s="2" t="n">
         <v>0</v>
@@ -5034,14 +5034,14 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>Intensivering 2026; niet in 2027.</t>
+          <t>Kost netto geld (minder naheffingen); geschrapt.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Schrappen cultuurprogramma Niemeyer (vervallen)</t>
+          <t>Preventiefonds jeugd (v1 als uitgave) (vervallen)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5059,7 +5059,7 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n">
-        <v>0.25</v>
+        <v>-4.509</v>
       </c>
       <c r="I87" s="2" t="n">
         <v>0</v>
@@ -5079,14 +5079,14 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>Intensivering 2026 (eenmalig); niet in 2027.</t>
+          <t>Fonds liep t/m 2026 (begroting 2026); bestaat in 2027 niet meer.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Stoppen uitvoering plan van aanpak diversiteit (vervallen)</t>
+          <t>Organisatiekosten Energiebedrijf Groningen (vervallen)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5104,7 +5104,7 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n">
-        <v>0.205</v>
+        <v>0.201</v>
       </c>
       <c r="I88" s="2" t="n">
         <v>0</v>
@@ -5131,7 +5131,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Ambtenaren gebiedsontwikkeling +5% (vervallen)</t>
+          <t>Schrappen cultuurprogramma Niemeyer (vervallen)</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -5149,7 +5149,7 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n">
-        <v>-0.35</v>
+        <v>0.25</v>
       </c>
       <c r="I89" s="2" t="n">
         <v>0</v>
@@ -5169,54 +5169,144 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
+          <t>Intensivering 2026 (eenmalig); niet in 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Stoppen uitvoering plan van aanpak diversiteit (vervallen)</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Ombuiging</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" s="2" t="n"/>
+      <c r="H90" s="2" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" s="2">
+        <f>I90-H90</f>
+        <v/>
+      </c>
+      <c r="K90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Intensivering 2026; niet in 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Ambtenaren gebiedsontwikkeling +5% (vervallen)</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Ombuiging</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" s="2" t="n"/>
+      <c r="H91" s="2" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" s="2">
+        <f>I91-H91</f>
+        <v/>
+      </c>
+      <c r="K91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
           <t>Geschrapt (fractiebesluit): past niet bij de vacaturestop.</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="3" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
         <is>
           <t>Saldo (+ = overschot)</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr"/>
-      <c r="C90" s="3" t="inlineStr"/>
-      <c r="D90" s="3" t="inlineStr"/>
-      <c r="E90" s="3" t="inlineStr"/>
-      <c r="F90" s="3" t="inlineStr"/>
-      <c r="G90" s="4" t="inlineStr"/>
-      <c r="H90" s="4">
-        <f>SUM(H2:H89)</f>
-        <v/>
-      </c>
-      <c r="I90" s="4">
-        <f>SUM(I2:I89)</f>
-        <v/>
-      </c>
-      <c r="J90" s="4">
-        <f>I90-H90</f>
-        <v/>
-      </c>
-      <c r="K90" s="4">
-        <f>SUM(K2:K89)</f>
-        <v/>
-      </c>
-      <c r="L90" s="4">
-        <f>SUM(L2:L89)</f>
-        <v/>
-      </c>
-      <c r="M90" s="4">
-        <f>SUM(M2:M89)</f>
-        <v/>
-      </c>
-      <c r="N90" s="3" t="inlineStr">
-        <is>
-          <t>v1: 51,475 (storting). Game: 11,786.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="B92" s="3" t="inlineStr"/>
+      <c r="C92" s="3" t="inlineStr"/>
+      <c r="D92" s="3" t="inlineStr"/>
+      <c r="E92" s="3" t="inlineStr"/>
+      <c r="F92" s="3" t="inlineStr"/>
+      <c r="G92" s="4" t="inlineStr"/>
+      <c r="H92" s="4">
+        <f>SUM(H2:H91)</f>
+        <v/>
+      </c>
+      <c r="I92" s="4">
+        <f>SUM(I2:I91)</f>
+        <v/>
+      </c>
+      <c r="J92" s="4">
+        <f>I92-H92</f>
+        <v/>
+      </c>
+      <c r="K92" s="4">
+        <f>SUM(K2:K91)</f>
+        <v/>
+      </c>
+      <c r="L92" s="4">
+        <f>SUM(L2:L91)</f>
+        <v/>
+      </c>
+      <c r="M92" s="4">
+        <f>SUM(M2:M91)</f>
+        <v/>
+      </c>
+      <c r="N92" s="3" t="inlineStr">
+        <is>
+          <t>v1: 51,475 (storting). Game: 11,381.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>Teken: + = gunstig voor het saldo (ombuiging/opbrengst), − = uitgave of kosten. Bedragen x 1 miljoen euro.</t>
         </is>
@@ -5558,16 +5648,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>13.839077</v>
+        <v>13.43366033333334</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>42.48325277319118</v>
+        <v>42.08258610652452</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>48.75215790990119</v>
+        <v>48.35624124323452</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>53.76009301243369</v>
+        <v>53.36892634576702</v>
       </c>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
@@ -5821,7 +5911,7 @@
         <v>-51.475</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-11.786477</v>
+        <v>-11.38106033333333</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>

</xml_diff>